<commit_message>
Merge latest version in main
</commit_message>
<xml_diff>
--- a/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260309.xlsx
+++ b/ssp_modeling/scenario_mapping/ssp_libya_transformation_cw_20260309.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10302"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="10308"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alexa/Projects/ssp_libya/ssp_modeling/scenario_mapping/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5098BE6-CD97-7549-9F4D-0E5FC71AD9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22F62445-40C1-BA40-AF22-30762F215089}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="80" yWindow="660" windowWidth="25340" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="main" sheetId="1" r:id="rId1"/>
     <sheet name="yaml" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$Q$64</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">main!$A$1:$R$64</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1">yaml!$A$1:$D$62</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="708" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="709" uniqueCount="413">
   <si>
     <t>subsector</t>
   </si>
@@ -1320,6 +1320,9 @@
   </si>
   <si>
     <t>transformation_enfu_adj_exports.yaml</t>
+  </si>
+  <si>
+    <t>strategy_Conditional</t>
   </si>
 </sst>
 </file>
@@ -1376,7 +1379,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1421,6 +1424,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1545,7 +1560,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="66">
+  <cellXfs count="71">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -1740,6 +1755,21 @@
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="9" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2047,24 +2077,24 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:Q64"/>
+  <dimension ref="A1:R64"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="13.1640625" style="36" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="43.5" style="36" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="5" style="36" customWidth="1"/>
-    <col min="5" max="5" width="9.33203125" style="36" customWidth="1"/>
+    <col min="4" max="4" width="32.1640625" style="36" customWidth="1"/>
+    <col min="5" max="5" width="23.83203125" style="36" customWidth="1"/>
     <col min="6" max="6" width="88.33203125" style="36" hidden="1" customWidth="1"/>
     <col min="7" max="10" width="13" style="36" hidden="1" customWidth="1"/>
     <col min="11" max="11" width="8" style="37" customWidth="1"/>
     <col min="12" max="12" width="5.83203125" style="38" customWidth="1"/>
-    <col min="13" max="14" width="20.5" style="39" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="13.5" style="40" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="13.5" style="39" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="13.5" style="41" bestFit="1" customWidth="1"/>
+    <col min="13" max="15" width="20.5" style="39" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5" style="40" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="13.5" style="39" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="13.5" style="41" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" s="4" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:18" s="4" customFormat="1" ht="65" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="5" t="s">
         <v>203</v>
       </c>
@@ -2104,14 +2134,17 @@
       <c r="M1" s="10" t="s">
         <v>407</v>
       </c>
-      <c r="N1" s="10" t="s">
+      <c r="N1" s="66" t="s">
         <v>212</v>
       </c>
-      <c r="O1" s="11"/>
-      <c r="P1" s="12"/>
+      <c r="O1" s="10" t="s">
+        <v>412</v>
+      </c>
+      <c r="P1" s="11"/>
       <c r="Q1" s="12"/>
-    </row>
-    <row r="2" spans="1:17" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R1" s="12"/>
+    </row>
+    <row r="2" spans="1:18" s="4" customFormat="1" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="13" t="s">
         <v>213</v>
       </c>
@@ -2142,14 +2175,15 @@
       </c>
       <c r="M2" s="18"/>
       <c r="N2" s="18"/>
-      <c r="O2" s="11">
+      <c r="O2" s="18"/>
+      <c r="P2" s="11">
         <f>K2*N2</f>
         <v>0</v>
       </c>
-      <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
-    </row>
-    <row r="3" spans="1:17" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R2" s="12"/>
+    </row>
+    <row r="3" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="13" t="s">
         <v>213</v>
       </c>
@@ -2180,14 +2214,15 @@
       </c>
       <c r="M3" s="18"/>
       <c r="N3" s="18"/>
-      <c r="O3" s="11">
-        <f t="shared" ref="O3:O8" si="0">K3*N3</f>
+      <c r="O3" s="18"/>
+      <c r="P3" s="11">
+        <f t="shared" ref="P3:P8" si="0">K3*N3</f>
         <v>0</v>
       </c>
-      <c r="P3" s="12"/>
       <c r="Q3" s="12"/>
-    </row>
-    <row r="4" spans="1:17" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R3" s="12"/>
+    </row>
+    <row r="4" spans="1:18" s="4" customFormat="1" ht="33" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="13" t="s">
         <v>213</v>
       </c>
@@ -2218,14 +2253,15 @@
       </c>
       <c r="M4" s="18"/>
       <c r="N4" s="18"/>
-      <c r="O4" s="11">
+      <c r="O4" s="18"/>
+      <c r="P4" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P4" s="12"/>
       <c r="Q4" s="12"/>
-    </row>
-    <row r="5" spans="1:17" s="4" customFormat="1" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R4" s="12"/>
+    </row>
+    <row r="5" spans="1:18" s="4" customFormat="1" ht="95.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="13" t="s">
         <v>213</v>
       </c>
@@ -2256,14 +2292,15 @@
       </c>
       <c r="M5" s="18"/>
       <c r="N5" s="18"/>
-      <c r="O5" s="11" t="e">
+      <c r="O5" s="18"/>
+      <c r="P5" s="11" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P5" s="12"/>
       <c r="Q5" s="12"/>
-    </row>
-    <row r="6" spans="1:17" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R5" s="12"/>
+    </row>
+    <row r="6" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="13" t="s">
         <v>213</v>
       </c>
@@ -2298,14 +2335,15 @@
       </c>
       <c r="M6" s="18"/>
       <c r="N6" s="18"/>
-      <c r="O6" s="11">
+      <c r="O6" s="18"/>
+      <c r="P6" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P6" s="12"/>
       <c r="Q6" s="12"/>
-    </row>
-    <row r="7" spans="1:17" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R6" s="12"/>
+    </row>
+    <row r="7" spans="1:18" s="4" customFormat="1" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="24" t="s">
         <v>227</v>
       </c>
@@ -2336,14 +2374,15 @@
       </c>
       <c r="M7" s="18"/>
       <c r="N7" s="18"/>
-      <c r="O7" s="11">
+      <c r="O7" s="18"/>
+      <c r="P7" s="11">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="P7" s="12"/>
       <c r="Q7" s="12"/>
-    </row>
-    <row r="8" spans="1:17" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R7" s="12"/>
+    </row>
+    <row r="8" spans="1:18" s="4" customFormat="1" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="13" t="s">
         <v>227</v>
       </c>
@@ -2353,7 +2392,7 @@
       <c r="C8" s="61" t="s">
         <v>25</v>
       </c>
-      <c r="D8" s="13" t="s">
+      <c r="D8" s="68" t="s">
         <v>26</v>
       </c>
       <c r="E8" s="13" t="s">
@@ -2376,20 +2415,21 @@
       <c r="L8" s="17">
         <v>12</v>
       </c>
-      <c r="M8" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M8" s="18"/>
       <c r="N8" s="18">
-        <v>1</v>
-      </c>
-      <c r="O8" s="11" t="e">
+        <v>0.05</v>
+      </c>
+      <c r="O8" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="P8" s="11" t="e">
         <f t="shared" si="0"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P8" s="12"/>
       <c r="Q8" s="12"/>
-    </row>
-    <row r="9" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R8" s="12"/>
+    </row>
+    <row r="9" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="13" t="s">
         <v>227</v>
       </c>
@@ -2424,14 +2464,15 @@
       </c>
       <c r="M9" s="18"/>
       <c r="N9" s="18"/>
-      <c r="O9" s="11">
+      <c r="O9" s="18"/>
+      <c r="P9" s="11">
         <f>K9*N9</f>
         <v>0</v>
       </c>
-      <c r="P9" s="12"/>
       <c r="Q9" s="12"/>
-    </row>
-    <row r="10" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R9" s="12"/>
+    </row>
+    <row r="10" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="13" t="s">
         <v>227</v>
       </c>
@@ -2441,7 +2482,7 @@
       <c r="C10" s="60" t="s">
         <v>31</v>
       </c>
-      <c r="D10" s="13" t="s">
+      <c r="D10" s="68" t="s">
         <v>32</v>
       </c>
       <c r="E10" s="13" t="s">
@@ -2464,20 +2505,21 @@
       <c r="L10" s="17">
         <v>12</v>
       </c>
-      <c r="M10" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M10" s="18"/>
       <c r="N10" s="18">
-        <v>1</v>
-      </c>
-      <c r="O10" s="11">
-        <f t="shared" ref="O10:O63" si="1">K10*N10</f>
-        <v>0.95</v>
-      </c>
-      <c r="P10" s="12"/>
+        <v>0.2</v>
+      </c>
+      <c r="O10" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P10" s="11">
+        <f t="shared" ref="P10:P63" si="1">K10*N10</f>
+        <v>0.19</v>
+      </c>
       <c r="Q10" s="12"/>
-    </row>
-    <row r="11" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R10" s="12"/>
+    </row>
+    <row r="11" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="13" t="s">
         <v>227</v>
       </c>
@@ -2487,7 +2529,7 @@
       <c r="C11" s="60" t="s">
         <v>35</v>
       </c>
-      <c r="D11" s="13" t="s">
+      <c r="D11" s="68" t="s">
         <v>36</v>
       </c>
       <c r="E11" s="13" t="s">
@@ -2506,20 +2548,21 @@
       <c r="L11" s="17">
         <v>12</v>
       </c>
-      <c r="M11" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M11" s="18"/>
       <c r="N11" s="18">
-        <v>1</v>
-      </c>
-      <c r="O11" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="O11" s="18">
+        <v>0.7</v>
+      </c>
+      <c r="P11" s="11">
         <f t="shared" si="1"/>
-        <v>0.8</v>
-      </c>
-      <c r="P11" s="12"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
       <c r="Q11" s="12"/>
-    </row>
-    <row r="12" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R11" s="12"/>
+    </row>
+    <row r="12" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A12" s="13" t="s">
         <v>227</v>
       </c>
@@ -2529,7 +2572,7 @@
       <c r="C12" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="D12" s="13" t="s">
+      <c r="D12" s="68" t="s">
         <v>39</v>
       </c>
       <c r="E12" s="13" t="s">
@@ -2548,20 +2591,21 @@
       <c r="L12" s="17">
         <v>12</v>
       </c>
-      <c r="M12" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M12" s="18"/>
       <c r="N12" s="18">
-        <v>1</v>
-      </c>
-      <c r="O12" s="11">
+        <v>0.05</v>
+      </c>
+      <c r="O12" s="18">
+        <v>0.7</v>
+      </c>
+      <c r="P12" s="11">
         <f t="shared" si="1"/>
-        <v>0.8</v>
-      </c>
-      <c r="P12" s="12"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
       <c r="Q12" s="12"/>
-    </row>
-    <row r="13" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R12" s="12"/>
+    </row>
+    <row r="13" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="13" t="s">
         <v>227</v>
       </c>
@@ -2571,7 +2615,7 @@
       <c r="C13" s="61" t="s">
         <v>42</v>
       </c>
-      <c r="D13" s="27" t="s">
+      <c r="D13" s="69" t="s">
         <v>43</v>
       </c>
       <c r="E13" s="27" t="s">
@@ -2594,20 +2638,21 @@
       <c r="L13" s="17">
         <v>12</v>
       </c>
-      <c r="M13" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M13" s="18"/>
       <c r="N13" s="18">
-        <v>1</v>
-      </c>
-      <c r="O13" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O13" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="P13" s="11">
         <f t="shared" si="1"/>
-        <v>0.3</v>
-      </c>
-      <c r="P13" s="12"/>
+        <v>0.03</v>
+      </c>
       <c r="Q13" s="12"/>
-    </row>
-    <row r="14" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R13" s="12"/>
+    </row>
+    <row r="14" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="13" t="s">
         <v>227</v>
       </c>
@@ -2617,7 +2662,7 @@
       <c r="C14" s="61" t="s">
         <v>45</v>
       </c>
-      <c r="D14" s="13" t="s">
+      <c r="D14" s="68" t="s">
         <v>46</v>
       </c>
       <c r="E14" s="13" t="s">
@@ -2640,20 +2685,21 @@
       <c r="L14" s="17">
         <v>12</v>
       </c>
-      <c r="M14" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M14" s="18"/>
       <c r="N14" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O14" s="18">
         <v>1</v>
       </c>
-      <c r="O14" s="11">
+      <c r="P14" s="11">
         <f t="shared" si="1"/>
-        <v>0.4</v>
-      </c>
-      <c r="P14" s="12"/>
+        <v>4.0000000000000008E-2</v>
+      </c>
       <c r="Q14" s="12"/>
-    </row>
-    <row r="15" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R14" s="12"/>
+    </row>
+    <row r="15" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="13" t="s">
         <v>227</v>
       </c>
@@ -2663,7 +2709,7 @@
       <c r="C15" s="61" t="s">
         <v>48</v>
       </c>
-      <c r="D15" s="13" t="s">
+      <c r="D15" s="68" t="s">
         <v>49</v>
       </c>
       <c r="E15" s="13" t="s">
@@ -2682,20 +2728,21 @@
       <c r="L15" s="17">
         <v>12</v>
       </c>
-      <c r="M15" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M15" s="18"/>
       <c r="N15" s="18">
-        <v>1</v>
-      </c>
-      <c r="O15" s="11" t="e">
+        <v>0.1</v>
+      </c>
+      <c r="O15" s="18">
+        <v>0.6</v>
+      </c>
+      <c r="P15" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P15" s="12"/>
       <c r="Q15" s="12"/>
-    </row>
-    <row r="16" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R15" s="12"/>
+    </row>
+    <row r="16" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="13" t="s">
         <v>51</v>
       </c>
@@ -2705,10 +2752,10 @@
       <c r="C16" s="61" t="s">
         <v>52</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="D16" s="68" t="s">
         <v>53</v>
       </c>
-      <c r="E16" s="13" t="s">
+      <c r="E16" s="61" t="s">
         <v>258</v>
       </c>
       <c r="F16" s="13" t="s">
@@ -2728,20 +2775,21 @@
       <c r="L16" s="17">
         <v>12</v>
       </c>
-      <c r="M16" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M16" s="18"/>
       <c r="N16" s="18">
-        <v>1.8</v>
-      </c>
-      <c r="O16" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O16" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="P16" s="11">
         <f t="shared" si="1"/>
-        <v>0.9</v>
-      </c>
-      <c r="P16" s="12"/>
+        <v>0.05</v>
+      </c>
       <c r="Q16" s="12"/>
-    </row>
-    <row r="17" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R16" s="12"/>
+    </row>
+    <row r="17" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="13" t="s">
         <v>51</v>
       </c>
@@ -2751,7 +2799,7 @@
       <c r="C17" s="13" t="s">
         <v>55</v>
       </c>
-      <c r="D17" s="27" t="s">
+      <c r="D17" s="69" t="s">
         <v>56</v>
       </c>
       <c r="E17" s="24" t="s">
@@ -2776,14 +2824,17 @@
       </c>
       <c r="M17" s="18"/>
       <c r="N17" s="18"/>
-      <c r="O17" s="11">
+      <c r="O17" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="P17" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P17" s="12"/>
       <c r="Q17" s="12"/>
-    </row>
-    <row r="18" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R17" s="12"/>
+    </row>
+    <row r="18" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="13" t="s">
         <v>51</v>
       </c>
@@ -2793,7 +2844,7 @@
       <c r="C18" s="61" t="s">
         <v>58</v>
       </c>
-      <c r="D18" s="13" t="s">
+      <c r="D18" s="68" t="s">
         <v>59</v>
       </c>
       <c r="E18" s="13" t="s">
@@ -2816,20 +2867,21 @@
       <c r="L18" s="17">
         <v>12</v>
       </c>
-      <c r="M18" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M18" s="18"/>
       <c r="N18" s="18">
-        <v>2</v>
-      </c>
-      <c r="O18" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O18" s="18">
+        <v>1</v>
+      </c>
+      <c r="P18" s="11">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="P18" s="12"/>
+        <v>1.0000000000000002E-2</v>
+      </c>
       <c r="Q18" s="12"/>
-    </row>
-    <row r="19" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R18" s="12"/>
+    </row>
+    <row r="19" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="13" t="s">
         <v>51</v>
       </c>
@@ -2839,10 +2891,10 @@
       <c r="C19" s="13" t="s">
         <v>61</v>
       </c>
-      <c r="D19" s="13" t="s">
+      <c r="D19" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="E19" s="13" t="s">
+      <c r="E19" s="67" t="s">
         <v>270</v>
       </c>
       <c r="F19" s="13" t="s">
@@ -2860,14 +2912,17 @@
       </c>
       <c r="M19" s="18"/>
       <c r="N19" s="18"/>
-      <c r="O19" s="11">
+      <c r="O19" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="P19" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P19" s="12"/>
       <c r="Q19" s="12"/>
-    </row>
-    <row r="20" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R19" s="12"/>
+    </row>
+    <row r="20" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A20" s="13" t="s">
         <v>51</v>
       </c>
@@ -2877,10 +2932,10 @@
       <c r="C20" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="D20" s="13" t="s">
+      <c r="D20" s="68" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="13" t="s">
+      <c r="E20" s="67" t="s">
         <v>272</v>
       </c>
       <c r="F20" s="13" t="s">
@@ -2898,14 +2953,17 @@
       </c>
       <c r="M20" s="18"/>
       <c r="N20" s="18"/>
-      <c r="O20" s="11">
+      <c r="O20" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="P20" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P20" s="12"/>
       <c r="Q20" s="12"/>
-    </row>
-    <row r="21" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R20" s="12"/>
+    </row>
+    <row r="21" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="13" t="s">
         <v>51</v>
       </c>
@@ -2915,10 +2973,10 @@
       <c r="C21" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="D21" s="13" t="s">
+      <c r="D21" s="68" t="s">
         <v>68</v>
       </c>
-      <c r="E21" s="13" t="s">
+      <c r="E21" s="67" t="s">
         <v>274</v>
       </c>
       <c r="F21" s="13" t="s">
@@ -2936,14 +2994,17 @@
       </c>
       <c r="M21" s="18"/>
       <c r="N21" s="18"/>
-      <c r="O21" s="11">
+      <c r="O21" s="18">
+        <v>0.5</v>
+      </c>
+      <c r="P21" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P21" s="12"/>
       <c r="Q21" s="12"/>
-    </row>
-    <row r="22" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R21" s="12"/>
+    </row>
+    <row r="22" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="13" t="s">
         <v>213</v>
       </c>
@@ -2978,14 +3039,15 @@
       </c>
       <c r="M22" s="18"/>
       <c r="N22" s="18"/>
-      <c r="O22" s="11">
+      <c r="O22" s="18"/>
+      <c r="P22" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P22" s="12"/>
       <c r="Q22" s="12"/>
-    </row>
-    <row r="23" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R22" s="12"/>
+    </row>
+    <row r="23" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="13" t="s">
         <v>213</v>
       </c>
@@ -3020,14 +3082,15 @@
       </c>
       <c r="M23" s="18"/>
       <c r="N23" s="18"/>
-      <c r="O23" s="11">
+      <c r="O23" s="18"/>
+      <c r="P23" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P23" s="12"/>
       <c r="Q23" s="12"/>
-    </row>
-    <row r="24" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R23" s="12"/>
+    </row>
+    <row r="24" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="13" t="s">
         <v>213</v>
       </c>
@@ -3037,7 +3100,7 @@
       <c r="C24" s="61" t="s">
         <v>77</v>
       </c>
-      <c r="D24" s="27" t="s">
+      <c r="D24" s="69" t="s">
         <v>78</v>
       </c>
       <c r="E24" s="24" t="s">
@@ -3060,20 +3123,21 @@
       <c r="L24" s="17">
         <v>12</v>
       </c>
-      <c r="M24" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M24" s="18"/>
       <c r="N24" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O24" s="18">
         <v>1</v>
       </c>
-      <c r="O24" s="11">
+      <c r="P24" s="11">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="P24" s="12"/>
+        <v>2.0000000000000004E-2</v>
+      </c>
       <c r="Q24" s="12"/>
-    </row>
-    <row r="25" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R24" s="12"/>
+    </row>
+    <row r="25" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="13" t="s">
         <v>213</v>
       </c>
@@ -3108,14 +3172,15 @@
       </c>
       <c r="M25" s="18"/>
       <c r="N25" s="18"/>
-      <c r="O25" s="11">
+      <c r="O25" s="18"/>
+      <c r="P25" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P25" s="12"/>
       <c r="Q25" s="12"/>
-    </row>
-    <row r="26" spans="1:17" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R25" s="12"/>
+    </row>
+    <row r="26" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="13" t="s">
         <v>213</v>
       </c>
@@ -3146,14 +3211,17 @@
       </c>
       <c r="M26" s="18"/>
       <c r="N26" s="18"/>
-      <c r="O26" s="11">
+      <c r="O26" s="18">
+        <v>0.4</v>
+      </c>
+      <c r="P26" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P26" s="12"/>
-      <c r="Q26" s="30"/>
-    </row>
-    <row r="27" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q26" s="12"/>
+      <c r="R26" s="30"/>
+    </row>
+    <row r="27" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="13" t="s">
         <v>213</v>
       </c>
@@ -3163,7 +3231,7 @@
       <c r="C27" s="60" t="s">
         <v>87</v>
       </c>
-      <c r="D27" s="13" t="s">
+      <c r="D27" s="68" t="s">
         <v>88</v>
       </c>
       <c r="E27" s="13" t="s">
@@ -3183,19 +3251,22 @@
         <v>12</v>
       </c>
       <c r="M27" s="18">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="N27" s="18">
-        <v>1</v>
-      </c>
-      <c r="O27" s="11" t="e">
+        <v>0.1</v>
+      </c>
+      <c r="O27" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P27" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P27" s="12"/>
       <c r="Q27" s="12"/>
-    </row>
-    <row r="28" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R27" s="12"/>
+    </row>
+    <row r="28" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A28" s="13" t="s">
         <v>213</v>
       </c>
@@ -3226,14 +3297,15 @@
       </c>
       <c r="M28" s="18"/>
       <c r="N28" s="18"/>
-      <c r="O28" s="11" t="e">
+      <c r="O28" s="18"/>
+      <c r="P28" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P28" s="12"/>
       <c r="Q28" s="12"/>
-    </row>
-    <row r="29" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R28" s="12"/>
+    </row>
+    <row r="29" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="13" t="s">
         <v>213</v>
       </c>
@@ -3264,14 +3336,15 @@
       </c>
       <c r="M29" s="18"/>
       <c r="N29" s="18"/>
-      <c r="O29" s="11" t="e">
+      <c r="O29" s="18"/>
+      <c r="P29" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P29" s="12"/>
       <c r="Q29" s="12"/>
-    </row>
-    <row r="30" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R29" s="12"/>
+    </row>
+    <row r="30" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="13" t="s">
         <v>213</v>
       </c>
@@ -3281,10 +3354,10 @@
       <c r="C30" s="60" t="s">
         <v>97</v>
       </c>
-      <c r="D30" s="13" t="s">
+      <c r="D30" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="E30" s="13" t="s">
+      <c r="E30" s="61" t="s">
         <v>301</v>
       </c>
       <c r="F30" s="13" t="s">
@@ -3301,19 +3374,22 @@
         <v>12</v>
       </c>
       <c r="M30" s="18">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="N30" s="18">
-        <v>1</v>
-      </c>
-      <c r="O30" s="11" t="e">
+        <v>0.1</v>
+      </c>
+      <c r="O30" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P30" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P30" s="12"/>
       <c r="Q30" s="12"/>
-    </row>
-    <row r="31" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R30" s="12"/>
+    </row>
+    <row r="31" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="13" t="s">
         <v>213</v>
       </c>
@@ -3344,14 +3420,15 @@
       </c>
       <c r="M31" s="18"/>
       <c r="N31" s="18"/>
-      <c r="O31" s="11">
+      <c r="O31" s="18"/>
+      <c r="P31" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P31" s="12"/>
       <c r="Q31" s="12"/>
-    </row>
-    <row r="32" spans="1:17" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R31" s="12"/>
+    </row>
+    <row r="32" spans="1:18" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="13" t="s">
         <v>213</v>
       </c>
@@ -3386,14 +3463,15 @@
       </c>
       <c r="M32" s="18"/>
       <c r="N32" s="18"/>
-      <c r="O32" s="11">
+      <c r="O32" s="18"/>
+      <c r="P32" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P32" s="18"/>
-      <c r="Q32" s="31"/>
-    </row>
-    <row r="33" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q32" s="18"/>
+      <c r="R32" s="31"/>
+    </row>
+    <row r="33" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="13" t="s">
         <v>310</v>
       </c>
@@ -3424,14 +3502,15 @@
       </c>
       <c r="M33" s="18"/>
       <c r="N33" s="18"/>
-      <c r="O33" s="11">
+      <c r="O33" s="18"/>
+      <c r="P33" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P33" s="12"/>
       <c r="Q33" s="12"/>
-    </row>
-    <row r="34" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R33" s="12"/>
+    </row>
+    <row r="34" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="13" t="s">
         <v>310</v>
       </c>
@@ -3462,14 +3541,15 @@
       </c>
       <c r="M34" s="18"/>
       <c r="N34" s="18"/>
-      <c r="O34" s="11">
+      <c r="O34" s="18"/>
+      <c r="P34" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P34" s="12"/>
       <c r="Q34" s="12"/>
-    </row>
-    <row r="35" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R34" s="12"/>
+    </row>
+    <row r="35" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="13" t="s">
         <v>227</v>
       </c>
@@ -3479,7 +3559,7 @@
       <c r="C35" s="60" t="s">
         <v>114</v>
       </c>
-      <c r="D35" s="13" t="s">
+      <c r="D35" s="68" t="s">
         <v>115</v>
       </c>
       <c r="E35" s="13" t="s">
@@ -3498,20 +3578,21 @@
       <c r="L35" s="17">
         <v>12</v>
       </c>
-      <c r="M35" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M35" s="18"/>
       <c r="N35" s="18">
-        <v>1</v>
-      </c>
-      <c r="O35" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O35" s="18">
+        <v>1.2</v>
+      </c>
+      <c r="P35" s="11">
         <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="P35" s="12"/>
+        <v>0.05</v>
+      </c>
       <c r="Q35" s="12"/>
-    </row>
-    <row r="36" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R35" s="12"/>
+    </row>
+    <row r="36" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A36" s="13" t="s">
         <v>227</v>
       </c>
@@ -3521,7 +3602,7 @@
       <c r="C36" s="61" t="s">
         <v>117</v>
       </c>
-      <c r="D36" s="13" t="s">
+      <c r="D36" s="68" t="s">
         <v>118</v>
       </c>
       <c r="E36" s="13" t="s">
@@ -3540,20 +3621,21 @@
       <c r="L36" s="17">
         <v>12</v>
       </c>
-      <c r="M36" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M36" s="18"/>
       <c r="N36" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O36" s="18">
         <v>1</v>
       </c>
-      <c r="O36" s="11">
+      <c r="P36" s="11">
         <f t="shared" si="1"/>
-        <v>0.5</v>
-      </c>
-      <c r="P36" s="12"/>
+        <v>0.05</v>
+      </c>
       <c r="Q36" s="12"/>
-    </row>
-    <row r="37" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R36" s="12"/>
+    </row>
+    <row r="37" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="13" t="s">
         <v>227</v>
       </c>
@@ -3563,7 +3645,7 @@
       <c r="C37" s="60" t="s">
         <v>120</v>
       </c>
-      <c r="D37" s="13" t="s">
+      <c r="D37" s="68" t="s">
         <v>121</v>
       </c>
       <c r="E37" s="13" t="s">
@@ -3582,20 +3664,21 @@
       <c r="L37" s="17">
         <v>12</v>
       </c>
-      <c r="M37" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M37" s="18"/>
       <c r="N37" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O37" s="18">
         <v>1</v>
       </c>
-      <c r="O37" s="11">
+      <c r="P37" s="11">
         <f t="shared" si="1"/>
-        <v>0.95</v>
-      </c>
-      <c r="P37" s="12"/>
+        <v>9.5000000000000001E-2</v>
+      </c>
       <c r="Q37" s="12"/>
-    </row>
-    <row r="38" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R37" s="12"/>
+    </row>
+    <row r="38" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="13" t="s">
         <v>213</v>
       </c>
@@ -3626,14 +3709,15 @@
       </c>
       <c r="M38" s="18"/>
       <c r="N38" s="18"/>
-      <c r="O38" s="11">
+      <c r="O38" s="18"/>
+      <c r="P38" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P38" s="12"/>
       <c r="Q38" s="12"/>
-    </row>
-    <row r="39" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R38" s="12"/>
+    </row>
+    <row r="39" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="13" t="s">
         <v>213</v>
       </c>
@@ -3643,7 +3727,7 @@
       <c r="C39" s="61" t="s">
         <v>127</v>
       </c>
-      <c r="D39" s="13" t="s">
+      <c r="D39" s="68" t="s">
         <v>128</v>
       </c>
       <c r="E39" s="13" t="s">
@@ -3662,20 +3746,21 @@
       <c r="L39" s="17">
         <v>12</v>
       </c>
-      <c r="M39" s="18">
+      <c r="M39" s="18"/>
+      <c r="N39" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O39" s="18">
         <v>0.5</v>
       </c>
-      <c r="N39" s="18">
-        <v>1</v>
-      </c>
-      <c r="O39" s="11">
+      <c r="P39" s="11">
         <f t="shared" si="1"/>
-        <v>0.2</v>
-      </c>
-      <c r="P39" s="12"/>
+        <v>2.0000000000000004E-2</v>
+      </c>
       <c r="Q39" s="12"/>
-    </row>
-    <row r="40" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R39" s="12"/>
+    </row>
+    <row r="40" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A40" s="13" t="s">
         <v>227</v>
       </c>
@@ -3685,7 +3770,7 @@
       <c r="C40" s="61" t="s">
         <v>131</v>
       </c>
-      <c r="D40" s="13" t="s">
+      <c r="D40" s="68" t="s">
         <v>132</v>
       </c>
       <c r="E40" s="13" t="s">
@@ -3708,20 +3793,21 @@
       <c r="L40" s="17">
         <v>12</v>
       </c>
-      <c r="M40" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M40" s="18"/>
       <c r="N40" s="18">
-        <v>1</v>
-      </c>
-      <c r="O40" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O40" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="P40" s="11">
         <f t="shared" si="1"/>
-        <v>0.25</v>
-      </c>
-      <c r="P40" s="12"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
       <c r="Q40" s="12"/>
-    </row>
-    <row r="41" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R40" s="12"/>
+    </row>
+    <row r="41" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="13" t="s">
         <v>227</v>
       </c>
@@ -3731,7 +3817,7 @@
       <c r="C41" s="61" t="s">
         <v>135</v>
       </c>
-      <c r="D41" s="13" t="s">
+      <c r="D41" s="68" t="s">
         <v>136</v>
       </c>
       <c r="E41" s="13" t="s">
@@ -3754,20 +3840,21 @@
       <c r="L41" s="17">
         <v>12</v>
       </c>
-      <c r="M41" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M41" s="18"/>
       <c r="N41" s="18">
-        <v>1</v>
-      </c>
-      <c r="O41" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O41" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="P41" s="11">
         <f t="shared" si="1"/>
-        <v>0.25</v>
-      </c>
-      <c r="P41" s="12"/>
+        <v>2.5000000000000001E-2</v>
+      </c>
       <c r="Q41" s="12"/>
-    </row>
-    <row r="42" spans="1:17" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R41" s="12"/>
+    </row>
+    <row r="42" spans="1:18" s="4" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A42" s="13" t="s">
         <v>227</v>
       </c>
@@ -3777,7 +3864,7 @@
       <c r="C42" s="61" t="s">
         <v>138</v>
       </c>
-      <c r="D42" s="13" t="s">
+      <c r="D42" s="68" t="s">
         <v>139</v>
       </c>
       <c r="E42" s="13" t="s">
@@ -3801,15 +3888,20 @@
         <v>12</v>
       </c>
       <c r="M42" s="18"/>
-      <c r="N42" s="18"/>
-      <c r="O42" s="11">
+      <c r="N42" s="18">
+        <v>0.05</v>
+      </c>
+      <c r="O42" s="18">
+        <v>1.5</v>
+      </c>
+      <c r="P42" s="11">
         <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-      <c r="P42" s="12"/>
+        <v>1.2500000000000001E-2</v>
+      </c>
       <c r="Q42" s="12"/>
-    </row>
-    <row r="43" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R42" s="12"/>
+    </row>
+    <row r="43" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="13" t="s">
         <v>227</v>
       </c>
@@ -3840,14 +3932,15 @@
       </c>
       <c r="M43" s="18"/>
       <c r="N43" s="18"/>
-      <c r="O43" s="11">
+      <c r="O43" s="18"/>
+      <c r="P43" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P43" s="12"/>
       <c r="Q43" s="12"/>
-    </row>
-    <row r="44" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R43" s="12"/>
+    </row>
+    <row r="44" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A44" s="13" t="s">
         <v>227</v>
       </c>
@@ -3857,7 +3950,7 @@
       <c r="C44" s="60" t="s">
         <v>144</v>
       </c>
-      <c r="D44" s="13" t="s">
+      <c r="D44" s="68" t="s">
         <v>145</v>
       </c>
       <c r="E44" s="13" t="s">
@@ -3876,20 +3969,21 @@
       <c r="L44" s="17">
         <v>12</v>
       </c>
-      <c r="M44" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M44" s="18"/>
       <c r="N44" s="18">
-        <v>1</v>
-      </c>
-      <c r="O44" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O44" s="18">
+        <v>0.8</v>
+      </c>
+      <c r="P44" s="11">
         <f t="shared" si="1"/>
-        <v>0.7</v>
-      </c>
-      <c r="P44" s="12"/>
+        <v>6.9999999999999993E-2</v>
+      </c>
       <c r="Q44" s="12"/>
-    </row>
-    <row r="45" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R44" s="12"/>
+    </row>
+    <row r="45" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="13" t="s">
         <v>227</v>
       </c>
@@ -3924,14 +4018,15 @@
       </c>
       <c r="M45" s="18"/>
       <c r="N45" s="18"/>
-      <c r="O45" s="11">
+      <c r="O45" s="18"/>
+      <c r="P45" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P45" s="12"/>
       <c r="Q45" s="12"/>
-    </row>
-    <row r="46" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R45" s="12"/>
+    </row>
+    <row r="46" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A46" s="13" t="s">
         <v>227</v>
       </c>
@@ -3941,7 +4036,7 @@
       <c r="C46" s="60" t="s">
         <v>150</v>
       </c>
-      <c r="D46" s="13" t="s">
+      <c r="D46" s="68" t="s">
         <v>151</v>
       </c>
       <c r="E46" s="13" t="s">
@@ -3964,20 +4059,21 @@
       <c r="L46" s="17">
         <v>12</v>
       </c>
-      <c r="M46" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M46" s="18"/>
       <c r="N46" s="18">
-        <v>1</v>
-      </c>
-      <c r="O46" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O46" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P46" s="11">
         <f t="shared" si="1"/>
-        <v>0.7</v>
-      </c>
-      <c r="P46" s="12"/>
+        <v>6.9999999999999993E-2</v>
+      </c>
       <c r="Q46" s="12"/>
-    </row>
-    <row r="47" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R46" s="12"/>
+    </row>
+    <row r="47" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="13" t="s">
         <v>227</v>
       </c>
@@ -4008,14 +4104,15 @@
       </c>
       <c r="M47" s="18"/>
       <c r="N47" s="18"/>
-      <c r="O47" s="11">
+      <c r="O47" s="18"/>
+      <c r="P47" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P47" s="12"/>
       <c r="Q47" s="12"/>
-    </row>
-    <row r="48" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R47" s="12"/>
+    </row>
+    <row r="48" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A48" s="13" t="s">
         <v>227</v>
       </c>
@@ -4050,14 +4147,15 @@
       </c>
       <c r="M48" s="18"/>
       <c r="N48" s="18"/>
-      <c r="O48" s="11">
+      <c r="O48" s="18"/>
+      <c r="P48" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P48" s="12"/>
       <c r="Q48" s="12"/>
-    </row>
-    <row r="49" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R48" s="12"/>
+    </row>
+    <row r="49" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="13" t="s">
         <v>227</v>
       </c>
@@ -4067,7 +4165,7 @@
       <c r="C49" s="61" t="s">
         <v>159</v>
       </c>
-      <c r="D49" s="13" t="s">
+      <c r="D49" s="68" t="s">
         <v>160</v>
       </c>
       <c r="E49" s="13" t="s">
@@ -4090,20 +4188,21 @@
       <c r="L49" s="17">
         <v>12</v>
       </c>
-      <c r="M49" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M49" s="18"/>
       <c r="N49" s="18">
-        <v>2</v>
-      </c>
-      <c r="O49" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O49" s="18">
+        <v>1</v>
+      </c>
+      <c r="P49" s="11">
         <f t="shared" si="1"/>
-        <v>0.6</v>
-      </c>
-      <c r="P49" s="12"/>
+        <v>0.03</v>
+      </c>
       <c r="Q49" s="12"/>
-    </row>
-    <row r="50" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R49" s="12"/>
+    </row>
+    <row r="50" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A50" s="13" t="s">
         <v>227</v>
       </c>
@@ -4138,14 +4237,15 @@
       </c>
       <c r="M50" s="18"/>
       <c r="N50" s="18"/>
-      <c r="O50" s="11" t="e">
+      <c r="O50" s="18"/>
+      <c r="P50" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P50" s="12"/>
       <c r="Q50" s="12"/>
-    </row>
-    <row r="51" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R50" s="12"/>
+    </row>
+    <row r="51" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="13" t="s">
         <v>51</v>
       </c>
@@ -4155,7 +4255,7 @@
       <c r="C51" s="61" t="s">
         <v>166</v>
       </c>
-      <c r="D51" s="13" t="s">
+      <c r="D51" s="68" t="s">
         <v>167</v>
       </c>
       <c r="E51" s="13" t="s">
@@ -4174,20 +4274,21 @@
       <c r="L51" s="17">
         <v>12</v>
       </c>
-      <c r="M51" s="18">
+      <c r="M51" s="18"/>
+      <c r="N51" s="18">
+        <v>0.1</v>
+      </c>
+      <c r="O51" s="18">
         <v>0.5</v>
       </c>
-      <c r="N51" s="18">
-        <v>1</v>
-      </c>
-      <c r="O51" s="11">
+      <c r="P51" s="11">
         <f t="shared" si="1"/>
-        <v>0.85</v>
-      </c>
-      <c r="P51" s="12"/>
+        <v>8.5000000000000006E-2</v>
+      </c>
       <c r="Q51" s="12"/>
-    </row>
-    <row r="52" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R51" s="12"/>
+    </row>
+    <row r="52" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A52" s="13" t="s">
         <v>51</v>
       </c>
@@ -4197,10 +4298,10 @@
       <c r="C52" s="13" t="s">
         <v>169</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="68" t="s">
         <v>170</v>
       </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="67" t="s">
         <v>366</v>
       </c>
       <c r="F52" s="13" t="s">
@@ -4222,14 +4323,17 @@
       </c>
       <c r="M52" s="18"/>
       <c r="N52" s="18"/>
-      <c r="O52" s="11">
+      <c r="O52" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="P52" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P52" s="12"/>
       <c r="Q52" s="12"/>
-    </row>
-    <row r="53" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R52" s="12"/>
+    </row>
+    <row r="53" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="13" t="s">
         <v>370</v>
       </c>
@@ -4264,14 +4368,15 @@
       </c>
       <c r="M53" s="18"/>
       <c r="N53" s="18"/>
-      <c r="O53" s="11" t="e">
+      <c r="O53" s="18"/>
+      <c r="P53" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P53" s="12"/>
       <c r="Q53" s="12"/>
-    </row>
-    <row r="54" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R53" s="12"/>
+    </row>
+    <row r="54" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A54" s="13" t="s">
         <v>370</v>
       </c>
@@ -4306,14 +4411,15 @@
       </c>
       <c r="M54" s="18"/>
       <c r="N54" s="18"/>
-      <c r="O54" s="11" t="e">
+      <c r="O54" s="18"/>
+      <c r="P54" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P54" s="12"/>
       <c r="Q54" s="12"/>
-    </row>
-    <row r="55" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R54" s="12"/>
+    </row>
+    <row r="55" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="13" t="s">
         <v>370</v>
       </c>
@@ -4323,7 +4429,7 @@
       <c r="C55" s="61" t="s">
         <v>179</v>
       </c>
-      <c r="D55" s="13" t="s">
+      <c r="D55" s="68" t="s">
         <v>180</v>
       </c>
       <c r="E55" s="13" t="s">
@@ -4347,19 +4453,22 @@
         <v>12</v>
       </c>
       <c r="M55" s="18">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="N55" s="18">
-        <v>1</v>
-      </c>
-      <c r="O55" s="11" t="e">
+        <v>0.1</v>
+      </c>
+      <c r="O55" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P55" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P55" s="12"/>
       <c r="Q55" s="12"/>
-    </row>
-    <row r="56" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R55" s="12"/>
+    </row>
+    <row r="56" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A56" s="13" t="s">
         <v>370</v>
       </c>
@@ -4369,7 +4478,7 @@
       <c r="C56" s="61" t="s">
         <v>183</v>
       </c>
-      <c r="D56" s="13" t="s">
+      <c r="D56" s="68" t="s">
         <v>184</v>
       </c>
       <c r="E56" s="13" t="s">
@@ -4392,20 +4501,21 @@
       <c r="L56" s="17">
         <v>12</v>
       </c>
-      <c r="M56" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M56" s="18"/>
       <c r="N56" s="18">
-        <v>1</v>
-      </c>
-      <c r="O56" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O56" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P56" s="11">
         <f t="shared" si="1"/>
-        <v>0.3</v>
-      </c>
-      <c r="P56" s="12"/>
+        <v>0.03</v>
+      </c>
       <c r="Q56" s="12"/>
-    </row>
-    <row r="57" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R56" s="12"/>
+    </row>
+    <row r="57" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="13" t="s">
         <v>370</v>
       </c>
@@ -4415,7 +4525,7 @@
       <c r="C57" s="61" t="s">
         <v>186</v>
       </c>
-      <c r="D57" s="13" t="s">
+      <c r="D57" s="68" t="s">
         <v>187</v>
       </c>
       <c r="E57" s="13" t="s">
@@ -4435,19 +4545,22 @@
         <v>12</v>
       </c>
       <c r="M57" s="18">
-        <v>0.5</v>
+        <v>0.1</v>
       </c>
       <c r="N57" s="18">
-        <v>1</v>
-      </c>
-      <c r="O57" s="11" t="e">
+        <v>0.1</v>
+      </c>
+      <c r="O57" s="18">
+        <v>0.3</v>
+      </c>
+      <c r="P57" s="11" t="e">
         <f t="shared" si="1"/>
         <v>#VALUE!</v>
       </c>
-      <c r="P57" s="12"/>
       <c r="Q57" s="12"/>
-    </row>
-    <row r="58" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R57" s="12"/>
+    </row>
+    <row r="58" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A58" s="13" t="s">
         <v>370</v>
       </c>
@@ -4457,7 +4570,7 @@
       <c r="C58" s="61" t="s">
         <v>189</v>
       </c>
-      <c r="D58" s="24" t="s">
+      <c r="D58" s="70" t="s">
         <v>167</v>
       </c>
       <c r="E58" s="24" t="s">
@@ -4480,20 +4593,21 @@
       <c r="L58" s="17">
         <v>12</v>
       </c>
-      <c r="M58" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M58" s="18"/>
       <c r="N58" s="18">
-        <v>1</v>
-      </c>
-      <c r="O58" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O58" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="P58" s="11">
         <f t="shared" si="1"/>
-        <v>0.85</v>
-      </c>
-      <c r="P58" s="12"/>
+        <v>8.5000000000000006E-2</v>
+      </c>
       <c r="Q58" s="12"/>
-    </row>
-    <row r="59" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R58" s="12"/>
+    </row>
+    <row r="59" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="13" t="s">
         <v>370</v>
       </c>
@@ -4503,7 +4617,7 @@
       <c r="C59" s="61" t="s">
         <v>191</v>
       </c>
-      <c r="D59" s="13" t="s">
+      <c r="D59" s="68" t="s">
         <v>192</v>
       </c>
       <c r="E59" s="13" t="s">
@@ -4522,20 +4636,21 @@
       <c r="L59" s="17">
         <v>12</v>
       </c>
-      <c r="M59" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M59" s="18"/>
       <c r="N59" s="18">
-        <v>1</v>
-      </c>
-      <c r="O59" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O59" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="P59" s="11">
         <f t="shared" si="1"/>
-        <v>0.85</v>
-      </c>
-      <c r="P59" s="12"/>
+        <v>8.5000000000000006E-2</v>
+      </c>
       <c r="Q59" s="12"/>
-    </row>
-    <row r="60" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R59" s="12"/>
+    </row>
+    <row r="60" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A60" s="13" t="s">
         <v>370</v>
       </c>
@@ -4545,7 +4660,7 @@
       <c r="C60" s="61" t="s">
         <v>194</v>
       </c>
-      <c r="D60" s="13" t="s">
+      <c r="D60" s="68" t="s">
         <v>195</v>
       </c>
       <c r="E60" s="13" t="s">
@@ -4564,20 +4679,21 @@
       <c r="L60" s="17">
         <v>12</v>
       </c>
-      <c r="M60" s="18">
-        <v>0.5</v>
-      </c>
+      <c r="M60" s="18"/>
       <c r="N60" s="18">
-        <v>1</v>
-      </c>
-      <c r="O60" s="11">
+        <v>0.1</v>
+      </c>
+      <c r="O60" s="18">
+        <v>0.2</v>
+      </c>
+      <c r="P60" s="11">
         <f t="shared" si="1"/>
-        <v>0.85</v>
-      </c>
-      <c r="P60" s="12"/>
+        <v>8.5000000000000006E-2</v>
+      </c>
       <c r="Q60" s="12"/>
-    </row>
-    <row r="61" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R60" s="12"/>
+    </row>
+    <row r="61" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="42" t="s">
         <v>370</v>
       </c>
@@ -4612,14 +4728,15 @@
       </c>
       <c r="M61" s="46"/>
       <c r="N61" s="46"/>
-      <c r="O61" s="11">
+      <c r="O61" s="46"/>
+      <c r="P61" s="11">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P61" s="12"/>
       <c r="Q61" s="12"/>
-    </row>
-    <row r="62" spans="1:17" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R61" s="12"/>
+    </row>
+    <row r="62" spans="1:18" s="4" customFormat="1" ht="85" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A62" s="47" t="s">
         <v>370</v>
       </c>
@@ -4654,14 +4771,15 @@
       </c>
       <c r="M62" s="51"/>
       <c r="N62" s="51"/>
-      <c r="O62" s="52">
+      <c r="O62" s="51"/>
+      <c r="P62" s="52">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P62" s="12"/>
       <c r="Q62" s="12"/>
-    </row>
-    <row r="63" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="R62" s="12"/>
+    </row>
+    <row r="63" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="48" t="s">
         <v>227</v>
       </c>
@@ -4688,14 +4806,15 @@
       </c>
       <c r="M63" s="53"/>
       <c r="N63" s="53"/>
-      <c r="O63" s="54">
+      <c r="O63" s="53"/>
+      <c r="P63" s="54">
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P63" s="12"/>
-      <c r="Q63" s="30"/>
-    </row>
-    <row r="64" spans="1:17" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="Q63" s="12"/>
+      <c r="R63" s="30"/>
+    </row>
+    <row r="64" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A64" s="33"/>
       <c r="B64" s="33"/>
       <c r="C64" s="33"/>
@@ -4710,13 +4829,14 @@
       <c r="L64" s="34"/>
       <c r="M64" s="12"/>
       <c r="N64" s="12"/>
-      <c r="O64" s="35"/>
-      <c r="P64" s="12"/>
-      <c r="Q64" s="29"/>
+      <c r="O64" s="12"/>
+      <c r="P64" s="35"/>
+      <c r="Q64" s="12"/>
+      <c r="R64" s="29"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q64" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
-  <conditionalFormatting sqref="M1:N1048576">
+  <autoFilter ref="A1:R64" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="M1:O1048576">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>

</xml_diff>